<commit_message>
docs(excel): Update Estrategias Global-Lubrikca xlsx and remove temporary Excel lock file
</commit_message>
<xml_diff>
--- a/Info_Odoo/Estrategias Global-Lubrikca. (1).xlsx
+++ b/Info_Odoo/Estrategias Global-Lubrikca. (1).xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Proyectos\CxC_Lubrikca\Info_Odoo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AF915B7-D2E7-45F1-9883-BACC3B3854C3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A1E1EA4E-5015-41CC-A979-9400A07859E4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="15600" windowHeight="11040" xr2:uid="{4E9660A1-968A-40F3-84DD-72ED71CADE3E}"/>
   </bookViews>
@@ -298,10 +298,10 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -628,29 +628,29 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>34</v>
       </c>
-      <c r="B1" s="16"/>
-      <c r="C1" s="16"/>
-      <c r="D1" s="16"/>
-      <c r="E1" s="16"/>
+      <c r="B1" s="17"/>
+      <c r="C1" s="17"/>
+      <c r="D1" s="17"/>
+      <c r="E1" s="17"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A2" s="17" t="s">
+      <c r="A2" s="16" t="s">
         <v>24</v>
       </c>
-      <c r="B2" s="17"/>
-      <c r="C2" s="17"/>
-      <c r="D2" s="17"/>
-      <c r="E2" s="17"/>
+      <c r="B2" s="16"/>
+      <c r="C2" s="16"/>
+      <c r="D2" s="16"/>
+      <c r="E2" s="16"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A3" s="16" t="s">
+      <c r="A3" s="17" t="s">
         <v>17</v>
       </c>
-      <c r="B3" s="16"/>
-      <c r="C3" s="16"/>
+      <c r="B3" s="17"/>
+      <c r="C3" s="17"/>
       <c r="D3" s="6" t="s">
         <v>44</v>
       </c>
@@ -693,11 +693,11 @@
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" s="16" t="s">
+      <c r="A6" s="17" t="s">
         <v>36</v>
       </c>
-      <c r="B6" s="16"/>
-      <c r="C6" s="16"/>
+      <c r="B6" s="17"/>
+      <c r="C6" s="17"/>
       <c r="D6" s="10"/>
       <c r="E6" s="10"/>
     </row>
@@ -736,11 +736,11 @@
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" s="16" t="s">
+      <c r="A9" s="17" t="s">
         <v>18</v>
       </c>
-      <c r="B9" s="16"/>
-      <c r="C9" s="16"/>
+      <c r="B9" s="17"/>
+      <c r="C9" s="17"/>
       <c r="D9" s="10"/>
       <c r="E9" s="10"/>
     </row>
@@ -867,11 +867,11 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="16" t="s">
+      <c r="A18" s="17" t="s">
         <v>19</v>
       </c>
-      <c r="B18" s="16"/>
-      <c r="C18" s="16"/>
+      <c r="B18" s="17"/>
+      <c r="C18" s="17"/>
       <c r="D18" s="10"/>
       <c r="E18" s="10"/>
     </row>
@@ -893,11 +893,11 @@
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" s="16" t="s">
+      <c r="A20" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="B20" s="16"/>
-      <c r="C20" s="16"/>
+      <c r="B20" s="17"/>
+      <c r="C20" s="17"/>
       <c r="D20" s="10"/>
       <c r="E20" s="10"/>
     </row>
@@ -922,22 +922,22 @@
       <c r="B22" s="1"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="17" t="s">
+      <c r="A23" s="16" t="s">
         <v>25</v>
       </c>
-      <c r="B23" s="17"/>
-      <c r="C23" s="17"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="17"/>
+      <c r="B23" s="16"/>
+      <c r="C23" s="16"/>
+      <c r="D23" s="16"/>
+      <c r="E23" s="16"/>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" s="16" t="s">
+      <c r="A24" s="17" t="s">
         <v>26</v>
       </c>
-      <c r="B24" s="16"/>
-      <c r="C24" s="16"/>
-      <c r="D24" s="16"/>
-      <c r="E24" s="16"/>
+      <c r="B24" s="17"/>
+      <c r="C24" s="17"/>
+      <c r="D24" s="17"/>
+      <c r="E24" s="17"/>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
@@ -957,13 +957,13 @@
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A26" s="16" t="s">
+      <c r="A26" s="17" t="s">
         <v>30</v>
       </c>
-      <c r="B26" s="16"/>
-      <c r="C26" s="16"/>
-      <c r="D26" s="16"/>
-      <c r="E26" s="16"/>
+      <c r="B26" s="17"/>
+      <c r="C26" s="17"/>
+      <c r="D26" s="17"/>
+      <c r="E26" s="17"/>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" s="15" t="s">
@@ -1035,9 +1035,7 @@
       <c r="A31" t="s">
         <v>51</v>
       </c>
-      <c r="B31" s="1">
-        <v>1</v>
-      </c>
+      <c r="B31" s="1"/>
       <c r="C31" t="s">
         <v>31</v>
       </c>
@@ -1100,11 +1098,11 @@
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A35" s="16" t="s">
+      <c r="A35" s="17" t="s">
         <v>21</v>
       </c>
-      <c r="B35" s="16"/>
-      <c r="C35" s="16"/>
+      <c r="B35" s="17"/>
+      <c r="C35" s="17"/>
       <c r="D35" s="10"/>
       <c r="E35" s="10"/>
     </row>
@@ -1127,17 +1125,17 @@
     </row>
   </sheetData>
   <mergeCells count="11">
-    <mergeCell ref="A2:E2"/>
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="A23:E23"/>
-    <mergeCell ref="A24:E24"/>
-    <mergeCell ref="A26:E26"/>
     <mergeCell ref="A35:C35"/>
     <mergeCell ref="A9:C9"/>
     <mergeCell ref="A6:C6"/>
     <mergeCell ref="A18:C18"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A23:E23"/>
+    <mergeCell ref="A24:E24"/>
+    <mergeCell ref="A26:E26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>

</xml_diff>